<commit_message>
"Fixed bugs and updated code"
</commit_message>
<xml_diff>
--- a/data/Appraisal Input.xlsx
+++ b/data/Appraisal Input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/int1961/Desktop/MyCareer-Agent-a-thon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDCF6F4D-9843-D545-B4C4-141A6D87DF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E7F69E-2E22-694B-AB3B-CD0F6354DA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -498,19 +498,10 @@
     <t>MMT1028</t>
   </si>
   <si>
-    <t>Gill</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Tree of Life turnaround followed by Taj West growth in H1, stands out as a remarkable success story, clearly reflecting the strongownershipandexecutionexcellence demonstrated by Nidhi.  Growing ToL from INR 2 Cr a year to 5 Cr a Qtr is highly commendable. </t>
   </si>
   <si>
-    <t xml:space="preserve">  Nidhi demonstrated aggressive execution with a strong  go-getter attitude , proactively taking  ownership  of tasks and driving them to closure with urgency and focus. This  bias for action  enables faster turnaround, improved execution quality, and tangible business outcomes. </t>
-  </si>
-  <si>
     <t>Inconsistency and a tendency toward delayed execution have been recurring feedback areas, where postponement of certain tasks has at times limited the desired business outcomes. We will work closely together to strengthen execution discipline and consistency, supporting her professional growth and overall impact</t>
-  </si>
-  <si>
-    <t>Nidhi has demonstrated strong partner relationship–building and effective communication skills, enabling her to collaborate seamlessly with stakeholders and drive alignment across engagements. Her ability to understand partner needs, manage expectations, and communicate clearly positions her well to take on broader responsibilities within supply roles across multiple lines of business.</t>
   </si>
   <si>
     <t>With continued exposure, she can add meaningful value by strengthening partnerships, improving execution, and supporting scalable growth across LOBs.</t>
@@ -1478,6 +1469,15 @@
   <si>
     <t>New to be considered.</t>
   </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Rahul demonstrated aggressive execution with a strong  go-getter attitude , proactively taking  ownership  of tasks and driving them to closure with urgency and focus. This  bias for action  enables faster turnaround, improved execution quality, and tangible business outcomes. </t>
+  </si>
+  <si>
+    <t>Rahul has demonstrated strong partner relationship–building and effective communication skills, enabling her to collaborate seamlessly with stakeholders and drive alignment across engagements. His ability to understand partner needs, manage expectations, and communicate clearly positions her well to take on broader responsibilities within supply roles across multiple lines of business.</t>
+  </si>
 </sst>
 </file>
 
@@ -1568,13 +1568,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2269,7 +2272,7 @@
       <c r="D14" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="4" t="s">
         <v>99</v>
       </c>
       <c r="F14" s="3" t="s">
@@ -2287,22 +2290,22 @@
         <v>101</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="F15" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>107</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>15</v>
@@ -2310,25 +2313,25 @@
     </row>
     <row r="16" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>114</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>15</v>
@@ -2336,25 +2339,25 @@
     </row>
     <row r="17" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>121</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>30</v>
@@ -2362,25 +2365,25 @@
     </row>
     <row r="18" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>125</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>128</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>60</v>
@@ -2388,25 +2391,25 @@
     </row>
     <row r="19" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="F19" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>132</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>135</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>15</v>
@@ -2414,25 +2417,25 @@
     </row>
     <row r="20" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="G20" s="3" t="s">
         <v>139</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>142</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>30</v>
@@ -2440,25 +2443,25 @@
     </row>
     <row r="21" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="F21" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="G21" s="3" t="s">
         <v>146</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>149</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>60</v>
@@ -2466,25 +2469,25 @@
     </row>
     <row r="22" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>153</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>156</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>15</v>
@@ -2492,25 +2495,25 @@
     </row>
     <row r="23" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>163</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>30</v>
@@ -2518,25 +2521,25 @@
     </row>
     <row r="24" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="F24" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="G24" s="3" t="s">
         <v>167</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>170</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>15</v>
@@ -2544,25 +2547,25 @@
     </row>
     <row r="25" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="E25" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="F25" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>176</v>
-      </c>
       <c r="G25" s="3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>60</v>
@@ -2570,25 +2573,25 @@
     </row>
     <row r="26" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="F26" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>182</v>
-      </c>
       <c r="G26" s="3" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>30</v>
@@ -2596,19 +2599,19 @@
     </row>
     <row r="27" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="E27" s="3" t="s">
         <v>184</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>187</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>67</v>
@@ -2622,25 +2625,25 @@
     </row>
     <row r="28" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="E28" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="G28" s="3" t="s">
         <v>191</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>194</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>30</v>
@@ -2648,25 +2651,25 @@
     </row>
     <row r="29" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="E29" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="F29" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="G29" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>201</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>60</v>
@@ -2674,25 +2677,25 @@
     </row>
     <row r="30" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="E30" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="F30" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="G30" s="3" t="s">
         <v>205</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>208</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>30</v>
@@ -2700,25 +2703,25 @@
     </row>
     <row r="31" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="F31" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="G31" s="3" t="s">
         <v>212</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>215</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>15</v>
@@ -2726,25 +2729,25 @@
     </row>
     <row r="32" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D32" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="E32" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="F32" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="G32" s="3" t="s">
         <v>219</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="G32" s="3" t="s">
-        <v>222</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>15</v>
@@ -2752,25 +2755,25 @@
     </row>
     <row r="33" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="D33" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="E33" s="3" t="s">
         <v>224</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>227</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>40</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>60</v>
@@ -2778,25 +2781,25 @@
     </row>
     <row r="34" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="D34" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="E34" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="F34" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="G34" s="3" t="s">
         <v>232</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="G34" s="3" t="s">
-        <v>235</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>15</v>
@@ -2804,25 +2807,25 @@
     </row>
     <row r="35" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="F35" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="G35" s="3" t="s">
         <v>239</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>242</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>15</v>
@@ -2830,25 +2833,25 @@
     </row>
     <row r="36" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="E36" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="F36" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="G36" s="3" t="s">
         <v>246</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>249</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>30</v>
@@ -2856,25 +2859,25 @@
     </row>
     <row r="37" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D37" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="E37" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="F37" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="G37" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>256</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>30</v>
@@ -2882,25 +2885,25 @@
     </row>
     <row r="38" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="D38" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="E38" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="F38" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="G38" s="3" t="s">
         <v>260</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>263</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>60</v>
@@ -2908,25 +2911,25 @@
     </row>
     <row r="39" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D39" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="E39" s="3" t="s">
         <v>265</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>268</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>67</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>30</v>
@@ -2934,25 +2937,25 @@
     </row>
     <row r="40" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="D40" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="E40" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="F40" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="G40" s="3" t="s">
         <v>273</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>276</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>60</v>
@@ -2960,25 +2963,25 @@
     </row>
     <row r="41" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="D41" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="E41" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="F41" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="D41" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>282</v>
-      </c>
       <c r="G41" s="3" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>30</v>
@@ -2986,25 +2989,25 @@
     </row>
     <row r="42" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="D42" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="E42" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="F42" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="G42" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>289</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>30</v>
@@ -3012,25 +3015,25 @@
     </row>
     <row r="43" spans="1:8" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="D43" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="E43" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="F43" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="D43" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>295</v>
-      </c>
       <c r="G43" s="3" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>30</v>

</xml_diff>